<commit_message>
final commit - all exp
</commit_message>
<xml_diff>
--- a/side_by_side_comparison.xlsx
+++ b/side_by_side_comparison.xlsx
@@ -1369,7 +1369,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>VALUE:12</t>
+          <t>VALUE:10</t>
         </is>
       </c>
       <c r="L15" t="b">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>HPE 1TB</t>
+          <t>HPE 1TB 6G SATA 7.2K rpm LFF (3.5in) Non-hot Plug Standard 1yr Warranty Hard Drive</t>
         </is>
       </c>
       <c r="L19" t="b">
@@ -1684,19 +1684,19 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>VALUE:2TB</t>
+          <t>L200</t>
         </is>
       </c>
       <c r="L20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>wrong</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" t="n">
         <v>3</v>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Aorus GeForce RTX 2060 Super</t>
+          <t>AORUS-GEFORCE-RTX-2060-SUPER</t>
         </is>
       </c>
       <c r="L26" t="b">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>130.0</t>
         </is>
       </c>
       <c r="L36" t="b">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="L37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>correct</t>
+          <t>wrong</t>
         </is>
       </c>
       <c r="N37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O37" t="n">
         <v>3</v>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>550</t>
         </is>
       </c>
       <c r="L41" t="b">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>22</t>
         </is>
       </c>
       <c r="L47" t="b">

</xml_diff>